<commit_message>
chore: sanitize docs and spreadsheet examples
</commit_message>
<xml_diff>
--- a/user.xlsx
+++ b/user.xlsx
@@ -31,11 +31,11 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
-    <t xml:space="preserve">说明：用户编号（工号，无工号填写身份证后8位）和姓名为必填；有效期截止格式如 20261231，留空默认为今天起10年；人脸图片名称需与user.xlsx表同文件夹内图片文件名一致；门填写门名称，多个门用英文逗号分隔；上传文件夹只读取user.xlsx文件，不要修改表名称；
-</t>
+    <t xml:space="preserve">说明：该文件为脱敏示例模板；用户编号和姓名为必填；有效期截止格式如 20261231；人脸图片名称请与同文件夹图片文件名一致；门字段多个值用英文逗号分隔；上传文件夹只读取 user.xlsx，请不要修改表名称。
+现有门名称示例：示例门禁1,示例门禁2,示例门禁3</t>
   </si>
   <si>
-    <t>现有门名称：传动轴大厅,传动轴2号人行门,传动轴3号人行门,传动轴10号人行门,传动轴11号人行门,传动轴12号人行门,传动轴成品库人行门,检验中心人行门,底零大厅,底零车间,底零2号人行门,底零6号人行门,底零7号人行门,底零8号人行门,部件联一大厅,部件联一10号人行门,部件联一11号人行门,部件联一12号人行门,部件联二24号人行门,部件联三27号人行门,部件联二28号人行门,部件联三25号人行门,部件联三26号人行门,部件联三27号人行门,部件联四20号人行门,部件联四23号人行门,部件冲压车间15号人行门,部件冲压车间19号人行门,部件冲压车间3楼,车轮大厅,精铸大厅,精铸大厅进车间</t>
+    <t>现有门名称示例：示例门禁1,示例门禁2,示例门禁3</t>
   </si>
   <si>
     <t>用户编号</t>
@@ -53,13 +53,13 @@
     <t>门</t>
   </si>
   <si>
-    <t>张三</t>
+    <t>示例用户</t>
   </si>
   <si>
-    <t>123.jpg</t>
+    <t>example_face.jpg</t>
   </si>
   <si>
-    <t>传动轴大厅,传动轴2号人行门</t>
+    <t>示例门禁1,示例门禁2</t>
   </si>
 </sst>
 </file>

</xml_diff>